<commit_message>
add research_area column and IaC paper to publications spreadsheet
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,6 +479,11 @@
           <t>doi</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>research_area</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -515,6 +520,11 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems,edge-and-on-device-ml</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -551,6 +561,11 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>miscellaneous</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -587,6 +602,11 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>edge-and-on-device-ml</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -627,6 +647,11 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -667,6 +692,11 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -707,6 +737,11 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -747,6 +782,11 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -787,6 +827,11 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>model-serving-and-inference</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -827,6 +872,11 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -867,6 +917,11 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>model-serving-and-inference</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -907,6 +962,11 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>miscellaneous</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -947,6 +1007,11 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -987,6 +1052,11 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1031,6 +1101,11 @@
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1075,6 +1150,11 @@
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems,edge-and-on-device-ml</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1119,6 +1199,11 @@
           <t>https://doi.org/10.1145/3664647.3681426</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1159,6 +1244,11 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1199,6 +1289,11 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1245,6 +1340,11 @@
       <c r="J20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1145/3643832.3661888</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>edge-and-on-device-ml</t>
         </is>
       </c>
     </row>
@@ -1287,6 +1387,11 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>model-serving-and-inference</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1335,6 +1440,11 @@
           <t>https://doi.org/10.1145/3627703.3650074</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>model-serving-and-inference</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1383,6 +1493,11 @@
           <t>https://doi.org/10.1145/3617232.3624849</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>model-serving-and-inference</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1427,6 +1542,11 @@
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems,edge-and-on-device-ml</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1471,6 +1591,11 @@
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>miscellaneous</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1511,6 +1636,11 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>edge-and-on-device-ml</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1551,6 +1681,11 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems,edge-and-on-device-ml</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1591,6 +1726,11 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>miscellaneous</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1635,6 +1775,11 @@
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1675,6 +1820,11 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>miscellaneous</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1715,6 +1865,11 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1759,6 +1914,11 @@
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1799,6 +1959,11 @@
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1847,6 +2012,11 @@
         </is>
       </c>
       <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1887,6 +2057,11 @@
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1931,6 +2106,11 @@
         </is>
       </c>
       <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1975,6 +2155,11 @@
         </is>
       </c>
       <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems,edge-and-on-device-ml</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2015,6 +2200,11 @@
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ai-for-systems</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2055,6 +2245,11 @@
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>model-serving-and-inference</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2095,6 +2290,11 @@
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2135,6 +2335,11 @@
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>miscellaneous</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2175,6 +2380,11 @@
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2215,6 +2425,11 @@
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>edge-and-on-device-ml</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2251,6 +2466,11 @@
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2291,6 +2511,11 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ai-for-systems</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2331,6 +2556,11 @@
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ai-for-systems</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2371,6 +2601,11 @@
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ai-for-systems</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2411,6 +2646,11 @@
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2451,6 +2691,11 @@
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2491,6 +2736,11 @@
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2531,6 +2781,11 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2571,6 +2826,11 @@
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2611,6 +2871,11 @@
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2651,6 +2916,11 @@
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2691,6 +2961,11 @@
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2731,6 +3006,11 @@
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ai-for-systems</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2771,6 +3051,11 @@
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2811,6 +3096,56 @@
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>miscellaneous</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Zhenning Yang, Hui Guan, Victor Nicolet, Brandon Paulsen, Joey Dodds, Daniel Kroening, Ang Chen</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Automated Cloud Infrastructure-as-Code Reconciliation with AI Agents</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>arXiv, 2025</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>arxiv25-iac-reconciliation</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2510.20211</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>arXiv'25</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>agentic-systems</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add missing ProTrain entry to spreadsheet with research_area
ProTrain (MLSys'26) existed as a hand-created publication file but was
missing from publications.xlsx. Added it with learning-algorithms-and-systems tag.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3147,6 +3147,51 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Hanmei Yang, Jin Zhou, Yao Fu, Xiaoquan Wang, Ramine Roane, Hui Guan, Tongping Liu</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ProTrain: Efficient LLM Training via Automatic Memory Management</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>The 9th Annual Conference on Machine Learning and Systems (MLSys 2026), Bellevue, WA, May 18-22, 2026</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>mlsys26-protrain-efficient</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2406.08334</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>MLSys'26</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>learning-algorithms-and-systems</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix broken CV page, missing TOP poster PDF link, and Dolby typo
- Remove cv.md which linked to nonexistent CV.pdf
- Clear paper_url for 2018 TOP poster (SysML'18) to remove broken PDF link
- Fix "Dobly" → "Dolby" typo in about.md
- Update intro text in about.md

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -511,15 +511,11 @@
           <t>sensys26-wildfit-autonomous</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>SenSys'26</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems,edge-and-on-device-ml</t>
@@ -552,15 +548,11 @@
           <t>pacificvis26-fourstage-framework</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>PacificVis'26</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>miscellaneous</t>
@@ -593,15 +585,11 @@
           <t>mmsys26-atom-efficient</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>MMSys'26</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>edge-and-on-device-ml</t>
@@ -644,9 +632,6 @@
           <t>VLDB'25</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -689,9 +674,6 @@
           <t>EXAIT@ICML'25</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -734,9 +716,6 @@
           <t>Neurocomputing@25</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -779,9 +758,6 @@
           <t>ARITH'25</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -824,9 +800,6 @@
           <t>TKDD'25</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>model-serving-and-inference</t>
@@ -869,9 +842,6 @@
           <t>MLSys'25</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -914,9 +884,6 @@
           <t>MLSys'25</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>model-serving-and-inference</t>
@@ -959,9 +926,6 @@
           <t>CHI EA'25</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>miscellaneous</t>
@@ -1004,9 +968,6 @@
           <t>MLforSys@NeurIPS'24</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -1049,9 +1010,6 @@
           <t>AI4Mat@NeurIPS'24</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -1099,8 +1057,6 @@
           <t>https://github.com/zhanglijun95/ZoDiac</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -1148,8 +1104,6 @@
           <t>https://github.com/Astuary/Spry</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems,edge-and-on-device-ml</t>
@@ -1192,8 +1146,6 @@
           <t>ACM MM'24</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>https://doi.org/10.1145/3664647.3681426</t>
@@ -1241,9 +1193,6 @@
           <t>MIPR'24</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -1286,9 +1235,6 @@
           <t>IEEE Access'24</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -1336,7 +1282,6 @@
           <t>https://github.com/mmehdirk/CACTUS-Dynamically-Switchable-Context-aware-micro-Classifiers-for-Efficient-IoT-Inference</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1145/3643832.3661888</t>
@@ -1384,9 +1329,6 @@
           <t>HPDC'24</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>model-serving-and-inference</t>
@@ -1434,7 +1376,6 @@
           <t>https://github.com/qizhengyang98/GMorph/tree/master</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>https://doi.org/10.1145/3627703.3650074</t>
@@ -1487,7 +1428,6 @@
           <t>https://github.com/UMass-LIDS/Proteus</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>https://doi.org/10.1145/3617232.3624849</t>
@@ -1540,8 +1480,6 @@
           <t>https://github.com/Astuary/Flow</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems,edge-and-on-device-ml</t>
@@ -1589,8 +1527,6 @@
           <t>https://zenodo.org/record/8350579</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>miscellaneous</t>
@@ -1633,9 +1569,6 @@
           <t>MobiCom'23</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
           <t>edge-and-on-device-ml</t>
@@ -1678,9 +1611,6 @@
           <t>ICML'23</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems,edge-and-on-device-ml</t>
@@ -1723,9 +1653,6 @@
           <t>ICML'23</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
           <t>miscellaneous</t>
@@ -1773,8 +1700,6 @@
           <t>https://github.com/zhanglijun95/TreeMTL</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -1817,9 +1742,6 @@
           <t>ISMM'23</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
           <t>miscellaneous</t>
@@ -1862,9 +1784,6 @@
           <t>IEEE Access'23</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -1912,8 +1831,6 @@
           <t>https://github.com/zhanglijun95/AutoMTL</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -1956,9 +1873,6 @@
           <t>VLDB'22</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2011,7 +1925,6 @@
           <t>Teaser~&gt;https://www.youtube.com/watch?v=t9r474WdBEQ|Video~&gt;https://www.youtube.com/watch?v=DobkdkBMFrg</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2054,9 +1967,6 @@
           <t>ICME'22</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2099,13 +2009,11 @@
           <t>AI4Science@ICML'22</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>talk~&gt;https://slideslive.com/38986179/improving-subgraph-representation-learning-via-multiview-augmentation</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2148,13 +2056,11 @@
           <t>CrossFL'22</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>Poster~&gt;https://crossfl2022.github.io/posters/Poster9.pdf</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems,edge-and-on-device-ml</t>
@@ -2197,9 +2103,6 @@
           <t>CGO'22</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
           <t>ai-for-systems</t>
@@ -2242,9 +2145,6 @@
           <t>ICDM'21</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
           <t>model-serving-and-inference</t>
@@ -2287,9 +2187,6 @@
           <t>OSR'21</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2332,9 +2229,6 @@
           <t>ICS'21</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
           <t>miscellaneous</t>
@@ -2377,9 +2271,6 @@
           <t>MCHPC'21</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2422,9 +2313,6 @@
           <t>CACM'21</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
           <t>edge-and-on-device-ml</t>
@@ -2457,15 +2345,11 @@
           <t>2021kmeans</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>InformationSystems'21</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2508,9 +2392,6 @@
           <t>CC'21</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>ai-for-systems</t>
@@ -2553,9 +2434,6 @@
           <t>FSE'20</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr">
         <is>
           <t>ai-for-systems</t>
@@ -2598,9 +2476,6 @@
           <t>TPDS'20</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
           <t>ai-for-systems</t>
@@ -2643,9 +2518,6 @@
           <t>MLSys'20</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2688,9 +2560,6 @@
           <t>NeurIPS'19</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2733,9 +2602,6 @@
           <t>MLSys@NeurIPS'19</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2778,9 +2644,6 @@
           <t>PLDI'19</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2823,9 +2686,6 @@
           <t>ICDE'19</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2868,9 +2728,6 @@
           <t>SC'18</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2913,9 +2770,6 @@
           <t>ICDE'18</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -2948,19 +2802,11 @@
           <t>2018top</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>http://guanh01.github.io/files/2018top.pdf</t>
-        </is>
-      </c>
       <c r="G55" t="inlineStr">
         <is>
           <t>SysML'18</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -3003,9 +2849,6 @@
           <t>SC'17</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
           <t>ai-for-systems</t>
@@ -3048,9 +2891,6 @@
           <t>PLDI'17</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>
@@ -3093,9 +2933,6 @@
           <t>SPAWC'16</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>miscellaneous</t>
@@ -3138,9 +2975,6 @@
           <t>arXiv'25</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
           <t>agentic-systems</t>
@@ -3183,9 +3017,6 @@
           <t>MLSys'26</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr">
         <is>
           <t>learning-algorithms-and-systems</t>

</xml_diff>